<commit_message>
Add example usage scripts and comprehensive tests for API functionality
- Created `ejemplos_uso.py` to demonstrate various API functionalities including simple queries, concurrent downloads, and handling multiple formats.
- Added `test_actualizacion.py` to verify imports, function signatures, request structures, and API endpoints.
- Implemented `test_api_response.py` to check the API response and validate MinIO fields.
- Developed `test_descarga_real.py` to simulate the complete download process, including CSV reading, directory creation, and file extraction.
</commit_message>
<xml_diff>
--- a/Descarga-Mis-Comprobantes.xlsx
+++ b/Descarga-Mis-Comprobantes.xlsx
@@ -49,13 +49,13 @@
     <t xml:space="preserve">Descarga Recibidos</t>
   </si>
   <si>
-    <t xml:space="preserve">Ubicación Emitidos</t>
+    <t xml:space="preserve">Ubicacion Emitidos</t>
   </si>
   <si>
     <t xml:space="preserve">Nombre Emitidos</t>
   </si>
   <si>
-    <t xml:space="preserve">Ubicación Recibidos</t>
+    <t xml:space="preserve">Ubicacion Recibidos</t>
   </si>
   <si>
     <t xml:space="preserve">Nombre Recibidos</t>

</xml_diff>